<commit_message>
Pulir entrega: numeración de páginas, hoja SE-01 y pendientes
Repaso contra las dos rúbricas para que no falte nada:

- Numeración de páginas en el pie de los dos documentos (la Tarea 4 la exige).
- Hoja completa de la sesión exploratoria SE-01, que antes solo se referenciaba;
  ahora el informe trae las dos hojas (SE-01 y SE-02), una por integrante.
- La evidencia de consola (F12) se enlaza también en los reportes de DEF-06 y
  DEF-10.
- La portada aclara cómo se gestionan las pruebas (repositorio ejecutable, con
  Qase como respaldo) y el README lista lo único que queda del equipo: firmas,
  enlaces, el contraste en Firefox y los dos casos de Google en Railway.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPYavKj2sG2dhvsf1XDSZo
</commit_message>
<xml_diff>
--- a/docs/entrega-2/E2_Registro_Ejecucion_EquipoF.xlsx
+++ b/docs/entrega-2/E2_Registro_Ejecucion_EquipoF.xlsx
@@ -3258,7 +3258,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>EV-DEF06-C1-01.png</t>
+          <t>EV-DEF06-C1-01.png, EV-DEF06-CONSOLA.png</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>EV-DEF10-C1-01.png</t>
+          <t>EV-DEF10-C1-01.png, EV-DEF10-CONSOLA.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerar evidencias y documentos con las capturas incrustadas
Corrida completa sobre base limpia (commit 693358a):
- Ciclo 1: 23 aprobados, 9 fallidos, 2 bloqueados (Google).
- Ciclo 2: 7 aprobados y los mismos 9 fallidos.
- Defectos exploratorios: DEF-05 verificado; DEF-06, 07, 10 y 14 abiertos.
- Consola F12: CP-008 (400), CP-018 (403), CP-021 (404) y los defectos
  DEF-06 (200), DEF-10 (201) y DEF-13 (inspección de #tostada).

E2_F_Equipo trae las 77 capturas como figuras: debajo de cada reporte
de defecto, en el Anexo D (consola) y en el nuevo Anexo E (ciclos 1 y 2).
La Tarea 4 trae las capturas de consola en el Anexo F y las de los ocho
defectos en el nuevo Anexo G, citadas por número de figura.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPYavKj2sG2dhvsf1XDSZo
</commit_message>
<xml_diff>
--- a/docs/entrega-2/E2_Registro_Ejecucion_EquipoF.xlsx
+++ b/docs/entrega-2/E2_Registro_Ejecucion_EquipoF.xlsx
@@ -851,7 +851,7 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:28 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:29 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:32 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:33 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:35 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:37 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:39 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:41 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:42 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:44 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:46 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:48 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:49 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:52 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:53 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:55 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:54 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:10:56 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:11:57 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:00 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:00 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:03 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:02 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:05 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:08 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:11 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:20 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:23 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:23 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:25 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:26 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:28 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:30 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:32 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:34 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:37 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:36 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:39 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:45 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:48 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:53 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:11:57 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>EV-CP021-C1-01.png</t>
+          <t>EV-CP021-C1-01.png, EV-CP021-C1-02.png</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:12:57 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:01 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:07 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:12 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:14 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:19 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Preparación: tutoría con Juan Salazar Bedoya el 08/10/2026 a las 04:13 (201); al pulsar «Cancelar» faltaban 12.0 h reales. PATCH → 400 {"error":"Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
+          <t>Preparación: tutoría con Juan Salazar Bedoya el 08/10/2026 a las 05:12 (201); al pulsar «Cancelar» faltaban 12.0 h reales. PATCH → 400 {"error":"Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:20 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:26 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Preparación: tutoría con Laura Vargas Suárez el 08/10/2026 a las 18:13 (201); al pulsar «Cancelar» faltaban 26.0 h reales. PATCH → 400 {"error":"Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
+          <t>Preparación: tutoría con Laura Vargas Suárez el 08/10/2026 a las 19:12 (201); al pulsar «Cancelar» faltaban 26.0 h reales. PATCH → 400 {"error":"Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:27 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:34 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:35 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:42 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:41 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:48 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:48 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:55 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>La primera fila es «07/10/2026 21:13 · admin.equipof@amigo.edu.co · 🔑 Login»: fecha legible y tipo correcto. El inicio de sesión se hizo a las 16:13 (hora de Colombia) y la tabla muestra 21:13: 5 horas de diferencia.</t>
+          <t>La primera fila es «07/10/2026 22:12 · admin.equipof@amigo.edu.co · 🔑 Login»: fecha legible y tipo correcto. El inicio de sesión se hizo a las 17:12 (hora de Colombia) y la tabla muestra 22:12: 5 horas de diferencia.</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:51 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:12:59 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>POST → 200 {"mensaje":"Enviado a 6 usuarios","cantidad":6}. La primera fila del historial es «07/10/2026 21:13 📅 Recordatorio de tutoría Todos los estudiantes en alerta (6) Recordatorio ✓ Enviado».</t>
+          <t>POST → 200 {"mensaje":"Enviado a 6 usuarios","cantidad":6}. La primera fila del historial es «07/10/2026 22:13 📅 Recordatorio de tutoría Todos los estudiantes en alerta (6) Recordatorio ✓ Enviado».</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:13:56 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:05 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:14:02 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:11 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>La asesoría con fecha de hoy (07/10/2026 18:11) se crea: POST → 200 {"mensaje":"Asesoría creada. Se notificó a Sandra Ríos Montoya y a Camilo Ríos Zapata.","tutoria_id":6}. Aparece en «Sesiones Programadas».</t>
+          <t>La asesoría con fecha de hoy (07/10/2026 19:10) se crea: POST → 200 {"mensaje":"Asesoría creada. Se notificó a Sandra Ríos Montoya y a Camilo Ríos Zapata.","tutoria_id":6}. Aparece en «Sesiones Programadas».</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:14:07 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:17 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:14:15 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:25 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:14:43 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:35 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:14:48 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:39 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:14:49 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:40 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:01 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:53 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:06 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:13:57 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:10 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:02 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:12 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:04 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:20 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:13 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:28 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:22 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>EV-CP021-C2-01.png</t>
+          <t>EV-CP021-C2-01.png, EV-CP021-C2-02.png</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:32 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:26 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:43 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:36 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>Preparación: tutoría con Juan Salazar Bedoya el 08/10/2026 a las 04:15 (201); al pulsar «Cancelar» faltaban 12.0 h reales. PATCH → 400 {"error":"Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
+          <t>Preparación: tutoría con Juan Salazar Bedoya el 08/10/2026 a las 05:14 (201); al pulsar «Cancelar» faltaban 12.0 h reales. PATCH → 400 {"error":"Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 7h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -2651,7 +2651,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:49 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:43 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>Preparación: tutoría con Laura Vargas Suárez el 08/10/2026 a las 18:15 (201); al pulsar «Cancelar» faltaban 26.0 h reales. PATCH → 400 {"error":"Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
+          <t>Preparación: tutoría con Laura Vargas Suárez el 08/10/2026 a las 19:14 (201); al pulsar «Cancelar» faltaban 26.0 h reales. PATCH → 400 {"error":"Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente."}; la tarjeta queda «Pendiente». En pantalla: el elemento #tostada tiene el texto «Faltan 21h para la tutoría y se requieren 24h de anticipación para cancelar (RN03). Escríbele al docente.» y las clases «tostada tostada--visible tostada--error», con opacidad calculada 0.</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:15:56 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:51 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:16:02 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:14:57 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>La asesoría con fecha de hoy (07/10/2026 18:14) se crea: POST → 200 {"mensaje":"Asesoría creada. Se notificó a Sandra Ríos Montoya y a Camilo Ríos Zapata.","tutoria_id":12}. Aparece en «Sesiones Programadas».</t>
+          <t>La asesoría con fecha de hoy (07/10/2026 19:13) se crea: POST → 200 {"mensaje":"Asesoría creada. Se notificó a Sandra Ríos Montoya y a Camilo Ríos Zapata.","tutoria_id":12}. Aparece en «Sesiones Programadas».</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:16:07 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:15:03 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>07/10/2026, 16:16:14 · Script E2 (Playwright)</t>
+          <t>07/10/2026, 17:15:11 · Script E2 (Playwright)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>EV-DEF06-C1-01.png, EV-DEF06-CONSOLA.png</t>
+          <t>EV-DEF06-C1-01.png, EV-DEF06-C1-02.png, EV-DEF06-C1-03.png, EV-DEF06-CONSOLA.png</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>EV-DEF10-C1-01.png, EV-DEF10-CONSOLA.png</t>
+          <t>EV-DEF10-C1-01.png, EV-DEF10-C1-02.png, EV-DEF10-CONSOLA.png</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3657,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>EV-CP016-C1-01.png</t>
+          <t>EV-CP016-C1-01.png, EV-CP024-C1-01.png, EV-DEF13-CONSOLA.png</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>EV-DEF14-C1-01.png</t>
+          <t>EV-DEF14-C1-01.png, EV-DEF14-C1-02.png</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar Anexo F para las capturas manuales en Railway (Google y Firefox)
- manual.json lista las 18 ejecuciones que hace el equipo a mano:
  CP-014 y CP-015 con Google y los 16 casos del ciclo 2 en Firefox,
  con quién las ejecuta y qué datos usar según la guía del equipo.
- El E2 trae una página por caso con su ficha y un recuadro punteado
  para pegar la captura en Word; si la captura ya está en
  resultados/manual/, se inserta como figura numerada.
- El registro xlsx suma la hoja «Manual en Railway» y agrega al
  registro las ejecuciones manuales que ya tengan captura y estado.
- El README explica dónde va cada captura y las dos formas de llenarlo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPYavKj2sG2dhvsf1XDSZo
</commit_message>
<xml_diff>
--- a/docs/entrega-2/E2_Registro_Ejecucion_EquipoF.xlsx
+++ b/docs/entrega-2/E2_Registro_Ejecucion_EquipoF.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro de ejecución" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reproducción cruzada" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Métricas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual en Railway" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reproducción cruzada" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Métricas" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Registro de ejecución'!$A$1:$H$51</definedName>
@@ -44,7 +45,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +70,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBEB"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +128,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2847,6 +2856,792 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Ciclo</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Lo ejecuta</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Qué se hace</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Estado esperado</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Estado obtenido</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Resultado real</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Navegador y versión</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Captura</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>CP-014</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Chrome o Firefox</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>En Railway, presionar «Continuar con Google» y entrar con una cuenta @amigo.edu.co.</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP014-RAILWAY.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>CP-015</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Chrome o Firefox</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>En Railway, presionar «Continuar con Google» y entrar con una cuenta @gmail.com.</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP015-RAILWAY.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>CP-007</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Sebastián González González</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Correo valido.c2@amigo.edu.co (si ya existe en Railway, valido.c3@amigo.edu.co).</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP007-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>CP-008</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Sebastián González González</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Correo admin.c2@amigo.edu.co, pegando el comando en la consola (F12).</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP008-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>CP-013</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Sebastián González González</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Cuenta nueva prueba.bloqueo3@amigo.edu.co.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP013-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>CP-016</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Cuenta nueva perfil.c2@amigo.edu.co.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP016-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>CP-017</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Otro estudiante, por ejemplo crios@amigo.edu.co.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP017-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>CP-018</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada; el comando se pega en la consola (F12).</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP018-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>CP-019</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada.</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP019-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>CP-020</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP020-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>CP-021</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada; el comando se pega en la consola (F12).</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP021-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>CP-022</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP022-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>CP-024</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Tutoría nueva con 12 horas de margen.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP024-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>CP-025</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Tutoría nueva con 26 horas de margen.</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP025-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>CP-031</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada.</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP031-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>CP-032</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Sebastián González González</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada (fecha de hoy).</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP032-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>CP-033</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Sebastián González González</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Fecha 02/04/2027.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP033-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>CP-034</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Esteban Palencia</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Railway · Firefox</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Repetir en Firefox, sobre Railway, los mismos pasos del ciclo 1. Datos: Nada.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Fallido</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>EV-CP034-FIREFOX.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3723,7 +4518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4149,7 +4944,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4164,204 +4959,204 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Métrica</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Meta del plan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Cobertura de requisitos</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>100 % (8 de 8)</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>100 %</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Casos diseñados</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Avance de ejecución · ciclo 1</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>32/34 ejecutables (100 %)</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>100 % de prioridad alta</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Aprobados · ciclo 1</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Se lee con el riesgo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Fallidos · ciclo 1</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Bloqueados · ciclo 1 (Google)</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Menos de 10 %</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Tasa de aprobación · ciclo 1</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>72 %</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Se lee con el riesgo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Tasa de aprobación · ciclo 2</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>44 %</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Se lee con el riesgo</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Defectos reportados</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>10 o más</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Defectos por severidad</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>1 crítica · 2 altas · 9 medias · 2 bajas</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Sin críticos abiertos</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Defectos verificados (corregidos)</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>1 de 14 (DEF-05)</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>